<commit_message>
feat: add archive management, reports, and system updates
</commit_message>
<xml_diff>
--- a/public/แพลตฟอร์มนำเข้าสินค้า.xlsx
+++ b/public/แพลตฟอร์มนำเข้าสินค้า.xlsx
@@ -3,9 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
-  </bookViews>
   <sheets>
     <sheet sheetId="1" name="ข้อมูลสินค้า" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="คำแนะนำ" state="visible" r:id="rId5"/>
@@ -15,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>แพลตฟอร์มนำเข้าสินค้า — ระบบ PIM</t>
   </si>
@@ -35,6 +32,9 @@
     <t>หมวดหมู่</t>
   </si>
   <si>
+    <t>หมวดหมู่ย่อย</t>
+  </si>
+  <si>
     <t>แบรนด์สินค้า</t>
   </si>
   <si>
@@ -80,50 +80,29 @@
     <t>วัตถุประสงค์</t>
   </si>
   <si>
-    <t>เทมเพลตนี้ใช้สำหรับกรอก/นำเข้าข้อมูลสินค้าให้ตรงกับโครงสร้างตาราง products ในระบบ PIM (Supabase)</t>
+    <t>เทมเพลตนี้ใช้สำหรับกรอก/นำเข้าข้อมูลสินค้าให้ตรงกับโครงสร้างระบบ PIM</t>
   </si>
   <si>
     <t>เริ่มกรอกที่แถว</t>
   </si>
   <si>
-    <t>แถวที่ 6 ของชีท "ข้อมูลสินค้า" (แถว 5 เป็นตัวอย่าง สีเหลือง ให้ลบทิ้งก่อนนำเข้าจริง)</t>
-  </si>
-  <si>
-    <t>รหัสสินค้า / รหัสบาร์โค้ด</t>
-  </si>
-  <si>
-    <t>ควรไม่ซ้ำกันในระบบ แนะนำกำหนดรูปแบบรหัสให้เป็นมาตรฐานเดียวกันทั้งไฟล์</t>
-  </si>
-  <si>
-    <t>ใส่เป็นลิงก์ URL รูปภาพ (หากยังไม่มีลิงก์ ให้เว้นว่างไว้ก่อน แล้วอัปโหลดผ่านหน้าเว็บภายหลัง)</t>
-  </si>
-  <si>
-    <t>เลือกจาก dropdown ได้เฉพาะ "ใช้งาน" หรือ "ไม่ใช้งาน" เท่านั้น</t>
-  </si>
-  <si>
-    <t>ราคาขายส่ง / ราคาขายปลีก / ค่าฝา</t>
-  </si>
-  <si>
-    <t>ต้องกรอกเป็นตัวเลขเท่านั้น (ห้ามใส่ตัวอักษรหรือสัญลักษณ์สกุลเงิน)</t>
-  </si>
-  <si>
-    <t>หมายเลข อย. / มอก.</t>
-  </si>
-  <si>
-    <t>หากไม่มีให้ใส่เครื่องหมาย - แทนการเว้นว่าง เพื่อป้องกันความสับสนว่าลืมกรอก</t>
-  </si>
-  <si>
-    <t>แถวสีเทาใต้หัวตาราง</t>
-  </si>
-  <si>
-    <t>เป็นชื่อฟิลด์ภายในระบบ (เช่น code, barcode) ไว้สำหรับอ้างอิงตอนนำเข้าเข้า Supabase ไม่ต้องแก้ไข</t>
+    <t>แถวที่ 3 ของชีท "ข้อมูลสินค้า"</t>
+  </si>
+  <si>
+    <t>หมวดหมู่ / หมวดหมู่ย่อย</t>
+  </si>
+  <si>
+    <t>กรอกหมวดหมู่หลักในช่องหมวดหมู่ และหมวดหมู่ย่อยในช่องหมวดหมู่ย่อย</t>
+  </si>
+  <si>
+    <t>กรอก "Active" หรือ "Inactive" (หรือ "เปิดใช้งาน" / "ปิดใช้งาน")</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -135,22 +114,13 @@
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="14"/>
-      <name val="Arial"/>
+      <name val="Sarabun"/>
     </font>
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
+      <name val="Sarabun"/>
     </font>
   </fonts>
   <fills count="4">
@@ -162,12 +132,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E78"/>
+        <fgColor rgb="FF1F497D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2E75B6"/>
+        <fgColor rgb="FF366092"/>
       </patternFill>
     </fill>
   </fills>
@@ -181,16 +151,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFB7B7B7"/>
+        <color rgb="FFB8CCE4"/>
       </left>
       <right style="thin">
-        <color rgb="FFB7B7B7"/>
+        <color rgb="FFB8CCE4"/>
       </right>
       <top style="thin">
-        <color rgb="FFB7B7B7"/>
+        <color rgb="FFB8CCE4"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFB7B7B7"/>
+        <color rgb="FFB8CCE4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -198,18 +168,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -303,6 +268,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -337,6 +303,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -371,20 +338,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -506,52 +469,91 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
+  <dimension ref="A1:R2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="40" customWidth="1"/>
-    <col min="5" max="6" width="18" customWidth="1"/>
-    <col min="7" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="14" customWidth="1"/>
-    <col min="15" max="15" width="40" customWidth="1"/>
-    <col min="16" max="17" width="35" customWidth="1"/>
+    <col min="4" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="13" width="15" customWidth="1"/>
+    <col min="14" max="14" width="12" customWidth="1"/>
+    <col min="15" max="15" width="15" customWidth="1"/>
+    <col min="16" max="18" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.95" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="35" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1"/>
-      <c r="C1"/>
-      <c r="D1"/>
-      <c r="E1"/>
-      <c r="F1"/>
-      <c r="G1"/>
-      <c r="H1"/>
-      <c r="I1"/>
-      <c r="J1"/>
-      <c r="K1"/>
-      <c r="L1"/>
-      <c r="M1"/>
-      <c r="N1"/>
-      <c r="O1"/>
-      <c r="P1"/>
-      <c r="Q1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
     </row>
-    <row r="2" ht="30" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" ht="28" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -602,112 +604,71 @@
       </c>
       <c r="Q2" s="2" t="s">
         <v>17</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
-  <dataValidations count="4">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="ค่าไม่ถูกต้อง" error="กรุณากรอกตัวเลขที่มากกว่าหรือเท่ากับ 0" sqref="K10:M1000">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="ค่าไม่ถูกต้อง" error="กรุณากรอกตัวเลขที่มากกว่าหรือเท่ากับ 0" sqref="K6:M1000">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="N10:N1000">
-      <formula1>"ใช้งาน,ไม่ใช้งาน"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="N6:N1000">
-      <formula1>"ใช้งาน,ไม่ใช้งาน"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="90" customWidth="1"/>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="75" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" t="s">
         <v>19</v>
       </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="2" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" s="5" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>21</v>
       </c>
+      <c r="B2" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="3" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" s="5" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>23</v>
       </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="4" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" s="5" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>25</v>
       </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="5" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="5" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: enhance product search with barcode auto-detect chips and update export stock labels
</commit_message>
<xml_diff>
--- a/public/แพลตฟอร์มนำเข้าสินค้า.xlsx
+++ b/public/แพลตฟอร์มนำเข้าสินค้า.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
   <si>
     <t>แพลตฟอร์มนำเข้าสินค้า — ระบบ PIM</t>
   </si>
@@ -44,6 +44,15 @@
     <t>น้ำหนัก</t>
   </si>
   <si>
+    <t>ความกว้างพัสดุ (ซม.)</t>
+  </si>
+  <si>
+    <t>ความยาวพัสดุ (ซม.)</t>
+  </si>
+  <si>
+    <t>ความสูงพัสดุ (ซม.)</t>
+  </si>
+  <si>
     <t>หมายเลข อย.</t>
   </si>
   <si>
@@ -93,6 +102,12 @@
   </si>
   <si>
     <t>กรอกหมวดหมู่หลักในช่องหมวดหมู่ และหมวดหมู่ย่อยในช่องหมวดหมู่ย่อย</t>
+  </si>
+  <si>
+    <t>ขนาดพัสดุ (กว้าง/ยาว/สูง)</t>
+  </si>
+  <si>
+    <t>กรอกเป็นตัวเลขหน่วยเซนติเมตร (ซม.) เช่น 10, 15, 20</t>
   </si>
   <si>
     <t>กรอก "Active" หรือ "Inactive" (หรือ "เปิดใช้งาน" / "ปิดใช้งาน")</t>
@@ -515,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -524,14 +539,14 @@
     <col min="4" max="6" width="25" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
     <col min="8" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="11" max="13" width="15" customWidth="1"/>
-    <col min="14" max="14" width="12" customWidth="1"/>
-    <col min="15" max="15" width="15" customWidth="1"/>
-    <col min="16" max="18" width="30" customWidth="1"/>
+    <col min="10" max="13" width="18" customWidth="1"/>
+    <col min="14" max="16" width="15" customWidth="1"/>
+    <col min="17" max="17" width="12" customWidth="1"/>
+    <col min="18" max="18" width="15" customWidth="1"/>
+    <col min="19" max="21" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="35" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -552,8 +567,11 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
     </row>
-    <row r="2" ht="28" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" ht="28" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -607,11 +625,20 @@
       </c>
       <c r="R2" s="2" t="s">
         <v>18</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A1:U1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -620,7 +647,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -629,42 +656,50 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>